<commit_message>
feat: highlight user custom items in light purple in Excel and hide unreviewed custom items from public master catalog
</commit_message>
<xml_diff>
--- a/출산준비물_통합데이터.xlsx
+++ b/출산준비물_통합데이터.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\.gemini\antigravity\scratch\kongkong\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\진규어플\출산준비물어플\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0BBBE05E-9B08-4B26-BAAF-254A162E7872}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B4675FD0-6914-440D-B3ED-4B13F6513AB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14415" activeTab="5" xr2:uid="{788198A8-8058-4D1A-8238-52DDCB41F95D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{02399CA1-EAED-454A-8052-CF66F4BDA800}"/>
   </bookViews>
   <sheets>
     <sheet name="출산가방 체크리스트" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,18 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -2785,7 +2797,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02C8DBF0-3492-48AF-92E6-1D1FFA7C9414}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFB3206B-F8A7-496B-9718-D983D49B3A71}">
   <dimension ref="A1:K64"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
@@ -4760,12 +4772,12 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2770643F-111E-4A5D-8616-80859450F545}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{399BC4B1-00D0-41C6-B792-3DBE4B49DD9B}">
   <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
@@ -5467,7 +5479,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16BB3175-6AFC-40CB-A530-D2B9F1E5D321}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79330AF7-82AD-483A-A056-402503BD0997}">
   <dimension ref="A1:E41"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
@@ -6182,7 +6194,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{667B3C2E-D9BA-4B3F-8DF3-50FFC17C28E3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A0545E3-D5BC-4E8A-BF28-4B0E5B5E1939}">
   <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
@@ -6567,7 +6579,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41CBCFD5-C905-4678-B6A1-827A44CDC5C1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F21E1C48-0AFE-4280-8099-C17C721D1BC6}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
@@ -6671,7 +6683,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1380B039-30BB-435A-94A7-17EB2A0D6656}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CA8445D-D70A-40AA-AA35-BA1340A1CAA9}">
   <dimension ref="A1:L1"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>

</xml_diff>

<commit_message>
feat(v1.1.4): reorder category chips with '전체' first and add/separate 12 essential bag items
</commit_message>
<xml_diff>
--- a/출산준비물_통합데이터.xlsx
+++ b/출산준비물_통합데이터.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\진규어플\출산준비물어플\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B571C13F-E898-485E-A8DE-F4757ABB75A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2EB126D0-4C70-4786-815D-FDE69C05E852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{6BD4DBDD-FDA2-49C9-9FA2-7748851977C3}"/>
+    <workbookView xWindow="5340" yWindow="3030" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="5" xr2:uid="{529BC0EA-11C5-48AB-B786-C56AF9AD1BF9}"/>
   </bookViews>
   <sheets>
     <sheet name="출산가방 체크리스트" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="806">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1257" uniqueCount="851">
   <si>
     <t>ID</t>
   </si>
@@ -566,7 +566,7 @@
     <t>개인 위생 &amp; 스킨케어</t>
   </si>
   <si>
-    <t>산모 세면도구 세트 (1세트)</t>
+    <t>산모 세면용품 세트 (1세트)</t>
   </si>
   <si>
     <t>(샴푸·바디워시·칫솔치약 등)</t>
@@ -644,6 +644,27 @@
     <t>콜라브 드라이샴푸 무향 저자극 파우더</t>
   </si>
   <si>
+    <t>m_sk_5</t>
+  </si>
+  <si>
+    <t>엄마용 영양제 (비타민, 철분 등)</t>
+  </si>
+  <si>
+    <t>1세트</t>
+  </si>
+  <si>
+    <t>(산후 회복·철분·비타민D·유산균)</t>
+  </si>
+  <si>
+    <t>솔가 철분 25mg 식물성 캡슐 (90일분)</t>
+  </si>
+  <si>
+    <t>닥터에디션 맘스 프로바이오틱스 유산균</t>
+  </si>
+  <si>
+    <t>종근당건강 락토핏 생유산균 맘스</t>
+  </si>
+  <si>
     <t>b_cloth_1</t>
   </si>
   <si>
@@ -866,6 +887,66 @@
     <t>말랑하니 유아 전동 손톱트리머</t>
   </si>
   <si>
+    <t>b_care_dday</t>
+  </si>
+  <si>
+    <t>디데이달력 (모자동실 성장 촬영용)</t>
+  </si>
+  <si>
+    <t>1개</t>
+  </si>
+  <si>
+    <t>(모자동실 기념사진 및 성장 기록)</t>
+  </si>
+  <si>
+    <t>말랑하니 아기 디데이달력 우드 스탠드형</t>
+  </si>
+  <si>
+    <t>달콤한기억 신생아 성장 디데이 캘린더</t>
+  </si>
+  <si>
+    <t>리틀포레스트 원목 감성 디데이달력</t>
+  </si>
+  <si>
+    <t>b_care_focusbook</t>
+  </si>
+  <si>
+    <t>초점책 (모자동실 흑백/컬러 초점책)</t>
+  </si>
+  <si>
+    <t>1권</t>
+  </si>
+  <si>
+    <t>(신생아 시각 발달 놀이용)</t>
+  </si>
+  <si>
+    <t>애플비 아기 초점책 병풍형 (흑백+컬러)</t>
+  </si>
+  <si>
+    <t>블루래빗 첫 두뇌계발 초점 플래시북</t>
+  </si>
+  <si>
+    <t>튤립사운드북 흑백 초점 병풍 세트</t>
+  </si>
+  <si>
+    <t>b_care_nightlight</t>
+  </si>
+  <si>
+    <t>수유등 (모자동실/조리원 밤 수유용)</t>
+  </si>
+  <si>
+    <t>(조도 조절 가능한 수유 무드등)</t>
+  </si>
+  <si>
+    <t>말랑하니 아기 무드등 LED 터치 수유등</t>
+  </si>
+  <si>
+    <t>바깃(Bagit) 모션인식 센서 터치 수유등</t>
+  </si>
+  <si>
+    <t>아르떼미데 톨로메오 미니 핀차 수유등</t>
+  </si>
+  <si>
     <t>b_safe_1</t>
   </si>
   <si>
@@ -1052,7 +1133,10 @@
     <t>g_dad_2</t>
   </si>
   <si>
-    <t>보호자 세면도구 &amp; 면도기</t>
+    <t>보호자(아빠) 세면용품 &amp; 면도기</t>
+  </si>
+  <si>
+    <t>(칫솔·치약·면도기·세안제)</t>
   </si>
   <si>
     <t>질레트 프로글라이드 플렉스볼 여행용 키트</t>
@@ -1085,10 +1169,10 @@
     <t>g_dad_4</t>
   </si>
   <si>
-    <t>보호자용 침구 / 이불 (필요시)</t>
-  </si>
-  <si>
-    <t>(보호자 침구 미제공 병원 확인)</t>
+    <t>아빠용 침구류 (이불·베개 / 필요시)</t>
+  </si>
+  <si>
+    <t>(병원 제공 여부 확인 필요)</t>
   </si>
   <si>
     <t>자주(JAJU) 접이식 극세사 캠핑 무릎담요</t>
@@ -1106,19 +1190,43 @@
     <t>생활 &amp; 편의 도구</t>
   </si>
   <si>
-    <t>구부러지는 꺾임 빨대 / 텀블러</t>
+    <t>텀블러 (보온/보냉용)</t>
+  </si>
+  <si>
+    <t>(손잡이형/빨대 호환)</t>
+  </si>
+  <si>
+    <t>스탠리 퀜처 H2.0 진공 텀블러</t>
+  </si>
+  <si>
+    <t>스탠리 퀜처 H2.0 플로우헤븐 진공 텀블러 887ml</t>
+  </si>
+  <si>
+    <t>글라스락 셰프토프 보온보냉 스트로우 텀블러</t>
+  </si>
+  <si>
+    <t>다이소 개별포장 주름 자바라 빨대 (100입)</t>
+  </si>
+  <si>
+    <t>g_life_straw</t>
+  </si>
+  <si>
+    <t>주름빨대 (구부러지는 꺾임 빨대)</t>
+  </si>
+  <si>
+    <t>1팩</t>
   </si>
   <si>
     <t>(누워서 수분 섭취 시 필수)</t>
   </si>
   <si>
-    <t>아띠빠스 실리콘 꺾임 빨대 텀블러 세트</t>
-  </si>
-  <si>
-    <t>글라스락 셰프토프 보온보냉 스트로우 텀블러</t>
-  </si>
-  <si>
-    <t>다이소 개별포장 주름 자바라 빨대 (100입)</t>
+    <t>다이소 개별포장 주름 자바라 꺾임빨대 (100입)</t>
+  </si>
+  <si>
+    <t>아띠빠스 실리콘 세척 가능 안심 꺾임 빨대</t>
+  </si>
+  <si>
+    <t>마더케이 일회용 꺾임 위생 빨대 60P</t>
   </si>
   <si>
     <t>g_life_2</t>
@@ -1136,25 +1244,43 @@
     <t>락앤락 메트로 머그 텀블러 600ml</t>
   </si>
   <si>
-    <t>g_life_3</t>
-  </si>
-  <si>
-    <t>스마트폰 충전기 &amp; 멀티탭 (3~5구)</t>
-  </si>
-  <si>
-    <t>(콘센트 거리 먼 경우 대비 2m 이상)</t>
+    <t>g_life_4</t>
+  </si>
+  <si>
+    <t>휴대폰 충전기 (긴 케이블 권장)</t>
+  </si>
+  <si>
+    <t>(침대 콘센트 거리 대비 2m 이상)</t>
   </si>
   <si>
     <t>벨킨 부스트업 초고속 3in1 멀티 충전기</t>
   </si>
   <si>
+    <t>신지모루 60W C타입 3미터 롱 케이블</t>
+  </si>
+  <si>
+    <t>삼성전자 45W 초고속 충전기 키트</t>
+  </si>
+  <si>
+    <t>g_life_multi</t>
+  </si>
+  <si>
+    <t>멀티탭 (3~5구, 긴 줄)</t>
+  </si>
+  <si>
+    <t>(산모 및 보호자 기기 동시 충전)</t>
+  </si>
+  <si>
+    <t>현대일렉트릭 서버탭 안전 멀티탭 4구 (3m)</t>
+  </si>
+  <si>
     <t>샤오미 멀티탭 3구 USB 3포트 (2m)</t>
   </si>
   <si>
-    <t>신지모루 60W C타입 3미터 롱 케이블</t>
-  </si>
-  <si>
-    <t>g_life_4</t>
+    <t>현대일렉트릭 고용량 개별 멀티탭 4구 (3m)</t>
+  </si>
+  <si>
+    <t>신성 개별 스위치 안전 멀티탭 5구</t>
   </si>
   <si>
     <t>휴대폰 거치대 (자바라/스탠드)</t>
@@ -1211,7 +1337,16 @@
     <t>g_life_7</t>
   </si>
   <si>
-    <t>손 소독제 &amp; 알코올 스왑</t>
+    <t>손세정제 (휴대용 손소독제)</t>
+  </si>
+  <si>
+    <t>(신생아 접촉 전 손 소독)</t>
+  </si>
+  <si>
+    <t>아이깨끗해 휴대용 거품형 손세정제</t>
+  </si>
+  <si>
+    <t>아이깨끗해 휴대용 거품형 손세정제 50ml</t>
   </si>
   <si>
     <t>유한양행 알코올 스왑 100매 개별포장</t>
@@ -1220,25 +1355,25 @@
     <t>데톨 오리지널 손소독 젤 200ml</t>
   </si>
   <si>
-    <t>닥터스에이 겔형 에탄올 손소독제</t>
-  </si>
-  <si>
-    <t>g_life_8</t>
-  </si>
-  <si>
-    <t>멀티 비타민 &amp; 철분제 &amp; 유산균</t>
-  </si>
-  <si>
-    <t>(산후 회복 및 수유 영양 보충)</t>
-  </si>
-  <si>
-    <t>솔가 철분 25mg 식물성 캡슐 (90일분)</t>
-  </si>
-  <si>
-    <t>닥터에디션 맘스 프로바이오틱스 유산균</t>
-  </si>
-  <si>
-    <t>종근당건강 락토핏 생유산균 베베/맘스</t>
+    <t>g_life_mask</t>
+  </si>
+  <si>
+    <t>일회용마스크 (KF94/비말 차단, 1팩)</t>
+  </si>
+  <si>
+    <t>(병원·조리원 방역 및 면회용)</t>
+  </si>
+  <si>
+    <t>아에르 KF94 피크 비말차단 마스크</t>
+  </si>
+  <si>
+    <t>아에르 KF94 피크 라이트 마스크 50매</t>
+  </si>
+  <si>
+    <t>크리넥스 데일리 비말차단 입체형 마스크 50매</t>
+  </si>
+  <si>
+    <t>웰킵스 뉴스마트 황사방역마스크 KF94 30매</t>
   </si>
   <si>
     <t>g_life_9</t>
@@ -2839,20 +2974,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F21FF587-FEC6-413E-929C-9470D5D53914}">
-  <dimension ref="A1:K64"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCF1F800-C143-404B-BD22-AF7A7E2C8C39}">
+  <dimension ref="A1:K70"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="1" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.25" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="34" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="40.75" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="45.625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="42.875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.75" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="44.125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="45.75" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="43.75" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="43.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3802,16 +3937,22 @@
         <v>200</v>
       </c>
       <c r="B32" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" t="s">
+        <v>173</v>
+      </c>
+      <c r="D32" t="s">
         <v>201</v>
       </c>
-      <c r="C32" t="s">
+      <c r="E32" t="s">
         <v>202</v>
       </c>
-      <c r="D32" t="s">
+      <c r="F32" t="s">
+        <v>15</v>
+      </c>
+      <c r="G32" t="s">
         <v>203</v>
-      </c>
-      <c r="F32" t="s">
-        <v>64</v>
       </c>
       <c r="H32" t="s">
         <v>204</v>
@@ -3831,193 +3972,190 @@
         <v>207</v>
       </c>
       <c r="B33" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C33" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="D33" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F33" t="s">
         <v>64</v>
       </c>
       <c r="H33" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="I33" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J33" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K33" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="34" spans="1:11">
       <c r="A34" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B34" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C34" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="D34" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F34" t="s">
         <v>64</v>
       </c>
-      <c r="G34" t="s">
-        <v>215</v>
-      </c>
       <c r="H34" t="s">
         <v>216</v>
       </c>
       <c r="I34" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J34" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K34" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="35" spans="1:11">
       <c r="A35" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B35" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C35" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="D35" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F35" t="s">
         <v>64</v>
       </c>
       <c r="G35" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H35" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I35" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J35" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K35" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="36" spans="1:11">
       <c r="A36" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B36" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C36" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="D36" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F36" t="s">
         <v>64</v>
       </c>
+      <c r="G36" t="s">
+        <v>228</v>
+      </c>
       <c r="H36" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="I36" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="J36" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="K36" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="37" spans="1:11">
       <c r="A37" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B37" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C37" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="D37" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="F37" t="s">
         <v>64</v>
       </c>
       <c r="H37" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="I37" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="J37" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="K37" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="38" spans="1:11">
       <c r="A38" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B38" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C38" t="s">
-        <v>236</v>
+        <v>209</v>
       </c>
       <c r="D38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F38" t="s">
-        <v>15</v>
-      </c>
-      <c r="G38" t="s">
-        <v>238</v>
+        <v>64</v>
       </c>
       <c r="H38" t="s">
         <v>239</v>
       </c>
       <c r="I38" t="s">
+        <v>239</v>
+      </c>
+      <c r="J38" t="s">
         <v>240</v>
       </c>
-      <c r="J38" t="s">
+      <c r="K38" t="s">
         <v>241</v>
-      </c>
-      <c r="K38" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="39" spans="1:11">
       <c r="A39" t="s">
+        <v>242</v>
+      </c>
+      <c r="B39" t="s">
+        <v>208</v>
+      </c>
+      <c r="C39" t="s">
         <v>243</v>
-      </c>
-      <c r="B39" t="s">
-        <v>201</v>
-      </c>
-      <c r="C39" t="s">
-        <v>236</v>
       </c>
       <c r="D39" t="s">
         <v>244</v>
@@ -4046,10 +4184,10 @@
         <v>250</v>
       </c>
       <c r="B40" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C40" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D40" t="s">
         <v>251</v>
@@ -4057,69 +4195,69 @@
       <c r="F40" t="s">
         <v>15</v>
       </c>
+      <c r="G40" t="s">
+        <v>252</v>
+      </c>
       <c r="H40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="I40" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="J40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K40" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="41" spans="1:11">
       <c r="A41" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B41" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C41" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D41" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F41" t="s">
         <v>15</v>
       </c>
       <c r="H41" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I41" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="J41" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="K41" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="42" spans="1:11">
       <c r="A42" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B42" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C42" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D42" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F42" t="s">
-        <v>167</v>
-      </c>
-      <c r="G42" t="s">
-        <v>263</v>
+        <v>15</v>
       </c>
       <c r="H42" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="I42" t="s">
         <v>265</v>
@@ -4136,10 +4274,10 @@
         <v>268</v>
       </c>
       <c r="B43" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C43" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D43" t="s">
         <v>269</v>
@@ -4147,150 +4285,162 @@
       <c r="F43" t="s">
         <v>167</v>
       </c>
+      <c r="G43" t="s">
+        <v>270</v>
+      </c>
       <c r="H43" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="I43" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="J43" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K43" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="44" spans="1:11">
       <c r="A44" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B44" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C44" t="s">
-        <v>275</v>
+        <v>243</v>
       </c>
       <c r="D44" t="s">
         <v>276</v>
       </c>
       <c r="F44" t="s">
-        <v>64</v>
-      </c>
-      <c r="G44" t="s">
+        <v>167</v>
+      </c>
+      <c r="H44" t="s">
         <v>277</v>
       </c>
-      <c r="H44" t="s">
+      <c r="I44" t="s">
         <v>278</v>
       </c>
-      <c r="I44" t="s">
+      <c r="J44" t="s">
         <v>279</v>
       </c>
-      <c r="J44" t="s">
+      <c r="K44" t="s">
         <v>280</v>
-      </c>
-      <c r="K44" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="45" spans="1:11">
       <c r="A45" t="s">
+        <v>281</v>
+      </c>
+      <c r="B45" t="s">
+        <v>208</v>
+      </c>
+      <c r="C45" t="s">
+        <v>243</v>
+      </c>
+      <c r="D45" t="s">
         <v>282</v>
       </c>
-      <c r="B45" t="s">
-        <v>201</v>
-      </c>
-      <c r="C45" t="s">
-        <v>275</v>
-      </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>283</v>
       </c>
       <c r="F45" t="s">
-        <v>64</v>
+        <v>167</v>
+      </c>
+      <c r="G45" t="s">
+        <v>284</v>
       </c>
       <c r="H45" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="I45" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="J45" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="K45" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="46" spans="1:11">
       <c r="A46" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B46" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C46" t="s">
-        <v>275</v>
+        <v>243</v>
       </c>
       <c r="D46" t="s">
-        <v>288</v>
+        <v>289</v>
+      </c>
+      <c r="E46" t="s">
+        <v>290</v>
       </c>
       <c r="F46" t="s">
         <v>167</v>
       </c>
       <c r="G46" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="H46" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="I46" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="J46" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="K46" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="47" spans="1:11">
       <c r="A47" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B47" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C47" t="s">
-        <v>275</v>
+        <v>243</v>
       </c>
       <c r="D47" t="s">
-        <v>294</v>
+        <v>296</v>
+      </c>
+      <c r="E47" t="s">
+        <v>283</v>
       </c>
       <c r="F47" t="s">
-        <v>64</v>
+        <v>15</v>
       </c>
       <c r="G47" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H47" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="I47" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J47" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="K47" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="48" spans="1:11">
       <c r="A48" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B48" t="s">
-        <v>301</v>
+        <v>208</v>
       </c>
       <c r="C48" t="s">
         <v>302</v>
@@ -4299,7 +4449,7 @@
         <v>303</v>
       </c>
       <c r="F48" t="s">
-        <v>15</v>
+        <v>64</v>
       </c>
       <c r="G48" t="s">
         <v>304</v>
@@ -4322,7 +4472,7 @@
         <v>309</v>
       </c>
       <c r="B49" t="s">
-        <v>301</v>
+        <v>208</v>
       </c>
       <c r="C49" t="s">
         <v>302</v>
@@ -4331,94 +4481,91 @@
         <v>310</v>
       </c>
       <c r="F49" t="s">
-        <v>15</v>
-      </c>
-      <c r="G49" t="s">
+        <v>64</v>
+      </c>
+      <c r="H49" t="s">
         <v>311</v>
       </c>
-      <c r="H49" t="s">
+      <c r="I49" t="s">
+        <v>311</v>
+      </c>
+      <c r="J49" t="s">
         <v>312</v>
       </c>
-      <c r="I49" t="s">
-        <v>312</v>
-      </c>
-      <c r="J49" t="s">
+      <c r="K49" t="s">
         <v>313</v>
-      </c>
-      <c r="K49" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="50" spans="1:11">
       <c r="A50" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B50" t="s">
-        <v>301</v>
+        <v>208</v>
       </c>
       <c r="C50" t="s">
         <v>302</v>
       </c>
       <c r="D50" t="s">
+        <v>315</v>
+      </c>
+      <c r="F50" t="s">
+        <v>167</v>
+      </c>
+      <c r="G50" t="s">
         <v>316</v>
       </c>
-      <c r="F50" t="s">
-        <v>15</v>
-      </c>
-      <c r="G50" t="s">
+      <c r="H50" t="s">
         <v>317</v>
       </c>
-      <c r="H50" t="s">
+      <c r="I50" t="s">
+        <v>317</v>
+      </c>
+      <c r="J50" t="s">
         <v>318</v>
       </c>
-      <c r="I50" t="s">
+      <c r="K50" t="s">
         <v>319</v>
-      </c>
-      <c r="J50" t="s">
-        <v>320</v>
-      </c>
-      <c r="K50" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="51" spans="1:11">
       <c r="A51" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B51" t="s">
-        <v>301</v>
+        <v>208</v>
       </c>
       <c r="C51" t="s">
         <v>302</v>
       </c>
       <c r="D51" t="s">
+        <v>321</v>
+      </c>
+      <c r="F51" t="s">
+        <v>64</v>
+      </c>
+      <c r="G51" t="s">
+        <v>322</v>
+      </c>
+      <c r="H51" t="s">
         <v>323</v>
       </c>
-      <c r="F51" t="s">
-        <v>167</v>
-      </c>
-      <c r="G51" t="s">
+      <c r="I51" t="s">
         <v>324</v>
       </c>
-      <c r="H51" t="s">
+      <c r="J51" t="s">
         <v>325</v>
       </c>
-      <c r="I51" t="s">
-        <v>325</v>
-      </c>
-      <c r="J51" t="s">
+      <c r="K51" t="s">
         <v>326</v>
-      </c>
-      <c r="K51" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="52" spans="1:11">
       <c r="A52" t="s">
+        <v>327</v>
+      </c>
+      <c r="B52" t="s">
         <v>328</v>
-      </c>
-      <c r="B52" t="s">
-        <v>301</v>
       </c>
       <c r="C52" t="s">
         <v>329</v>
@@ -4429,386 +4576,593 @@
       <c r="F52" t="s">
         <v>15</v>
       </c>
+      <c r="G52" t="s">
+        <v>331</v>
+      </c>
       <c r="H52" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="I52" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J52" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="K52" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="53" spans="1:11">
       <c r="A53" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B53" t="s">
-        <v>301</v>
+        <v>328</v>
       </c>
       <c r="C53" t="s">
         <v>329</v>
       </c>
       <c r="D53" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F53" t="s">
         <v>15</v>
       </c>
+      <c r="G53" t="s">
+        <v>338</v>
+      </c>
       <c r="H53" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="I53" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="J53" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K53" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="54" spans="1:11">
       <c r="A54" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B54" t="s">
-        <v>301</v>
+        <v>328</v>
       </c>
       <c r="C54" t="s">
         <v>329</v>
       </c>
       <c r="D54" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F54" t="s">
         <v>15</v>
       </c>
+      <c r="G54" t="s">
+        <v>344</v>
+      </c>
       <c r="H54" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="I54" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="J54" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="K54" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
     </row>
     <row r="55" spans="1:11">
       <c r="A55" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B55" t="s">
-        <v>301</v>
+        <v>328</v>
       </c>
       <c r="C55" t="s">
         <v>329</v>
       </c>
       <c r="D55" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="F55" t="s">
-        <v>194</v>
+        <v>167</v>
       </c>
       <c r="G55" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="H55" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="I55" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="J55" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="K55" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="56" spans="1:11">
       <c r="A56" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="B56" t="s">
-        <v>301</v>
+        <v>328</v>
       </c>
       <c r="C56" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="D56" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="F56" t="s">
         <v>15</v>
       </c>
-      <c r="G56" t="s">
-        <v>355</v>
-      </c>
       <c r="H56" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="I56" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="J56" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="K56" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="57" spans="1:11">
       <c r="A57" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B57" t="s">
-        <v>301</v>
+        <v>328</v>
       </c>
       <c r="C57" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="D57" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="F57" t="s">
         <v>15</v>
       </c>
+      <c r="G57" t="s">
+        <v>364</v>
+      </c>
       <c r="H57" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="I57" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="J57" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="K57" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
     </row>
     <row r="58" spans="1:11">
       <c r="A58" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="B58" t="s">
-        <v>301</v>
+        <v>328</v>
       </c>
       <c r="C58" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="D58" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="F58" t="s">
         <v>15</v>
       </c>
-      <c r="G58" t="s">
-        <v>366</v>
-      </c>
       <c r="H58" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="I58" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="J58" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="K58" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
     </row>
     <row r="59" spans="1:11">
       <c r="A59" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="B59" t="s">
-        <v>301</v>
+        <v>328</v>
       </c>
       <c r="C59" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="D59" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="F59" t="s">
-        <v>15</v>
+        <v>194</v>
       </c>
       <c r="G59" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="H59" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="I59" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="J59" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="K59" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
     </row>
     <row r="60" spans="1:11">
       <c r="A60" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="B60" t="s">
-        <v>301</v>
+        <v>328</v>
       </c>
       <c r="C60" t="s">
-        <v>353</v>
+        <v>381</v>
       </c>
       <c r="D60" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="F60" t="s">
         <v>15</v>
       </c>
+      <c r="G60" t="s">
+        <v>383</v>
+      </c>
       <c r="H60" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="I60" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="J60" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="K60" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
     </row>
     <row r="61" spans="1:11">
       <c r="A61" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="B61" t="s">
-        <v>301</v>
+        <v>328</v>
       </c>
       <c r="C61" t="s">
-        <v>353</v>
+        <v>381</v>
       </c>
       <c r="D61" t="s">
-        <v>383</v>
+        <v>389</v>
+      </c>
+      <c r="E61" t="s">
+        <v>390</v>
       </c>
       <c r="F61" t="s">
         <v>15</v>
       </c>
       <c r="G61" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="H61" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="I61" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="J61" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="K61" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
     </row>
     <row r="62" spans="1:11">
       <c r="A62" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="B62" t="s">
-        <v>301</v>
+        <v>328</v>
       </c>
       <c r="C62" t="s">
-        <v>353</v>
+        <v>381</v>
       </c>
       <c r="D62" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="F62" t="s">
         <v>15</v>
       </c>
       <c r="H62" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="I62" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="J62" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="K62" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
     </row>
     <row r="63" spans="1:11">
       <c r="A63" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="B63" t="s">
-        <v>301</v>
+        <v>328</v>
       </c>
       <c r="C63" t="s">
-        <v>353</v>
+        <v>381</v>
       </c>
       <c r="D63" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="F63" t="s">
         <v>15</v>
       </c>
       <c r="G63" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="H63" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="I63" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="J63" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="K63" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
     </row>
     <row r="64" spans="1:11">
       <c r="A64" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="B64" t="s">
-        <v>301</v>
+        <v>328</v>
       </c>
       <c r="C64" t="s">
-        <v>353</v>
+        <v>381</v>
       </c>
       <c r="D64" t="s">
-        <v>400</v>
+        <v>407</v>
+      </c>
+      <c r="E64" t="s">
+        <v>283</v>
       </c>
       <c r="F64" t="s">
         <v>15</v>
       </c>
       <c r="G64" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="H64" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="I64" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="J64" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="K64" t="s">
-        <v>404</v>
+        <v>412</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11">
+      <c r="A65" t="s">
+        <v>400</v>
+      </c>
+      <c r="B65" t="s">
+        <v>328</v>
+      </c>
+      <c r="C65" t="s">
+        <v>381</v>
+      </c>
+      <c r="D65" t="s">
+        <v>413</v>
+      </c>
+      <c r="F65" t="s">
+        <v>15</v>
+      </c>
+      <c r="G65" t="s">
+        <v>414</v>
+      </c>
+      <c r="H65" t="s">
+        <v>415</v>
+      </c>
+      <c r="I65" t="s">
+        <v>415</v>
+      </c>
+      <c r="J65" t="s">
+        <v>416</v>
+      </c>
+      <c r="K65" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11">
+      <c r="A66" t="s">
+        <v>418</v>
+      </c>
+      <c r="B66" t="s">
+        <v>328</v>
+      </c>
+      <c r="C66" t="s">
+        <v>381</v>
+      </c>
+      <c r="D66" t="s">
+        <v>419</v>
+      </c>
+      <c r="F66" t="s">
+        <v>15</v>
+      </c>
+      <c r="H66" t="s">
+        <v>420</v>
+      </c>
+      <c r="I66" t="s">
+        <v>421</v>
+      </c>
+      <c r="J66" t="s">
+        <v>422</v>
+      </c>
+      <c r="K66" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11">
+      <c r="A67" t="s">
+        <v>424</v>
+      </c>
+      <c r="B67" t="s">
+        <v>328</v>
+      </c>
+      <c r="C67" t="s">
+        <v>381</v>
+      </c>
+      <c r="D67" t="s">
+        <v>425</v>
+      </c>
+      <c r="F67" t="s">
+        <v>15</v>
+      </c>
+      <c r="G67" t="s">
+        <v>426</v>
+      </c>
+      <c r="H67" t="s">
+        <v>427</v>
+      </c>
+      <c r="I67" t="s">
+        <v>427</v>
+      </c>
+      <c r="J67" t="s">
+        <v>428</v>
+      </c>
+      <c r="K67" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11">
+      <c r="A68" t="s">
+        <v>430</v>
+      </c>
+      <c r="B68" t="s">
+        <v>328</v>
+      </c>
+      <c r="C68" t="s">
+        <v>381</v>
+      </c>
+      <c r="D68" t="s">
+        <v>431</v>
+      </c>
+      <c r="F68" t="s">
+        <v>15</v>
+      </c>
+      <c r="G68" t="s">
+        <v>432</v>
+      </c>
+      <c r="H68" t="s">
+        <v>433</v>
+      </c>
+      <c r="I68" t="s">
+        <v>434</v>
+      </c>
+      <c r="J68" t="s">
+        <v>435</v>
+      </c>
+      <c r="K68" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11">
+      <c r="A69" t="s">
+        <v>437</v>
+      </c>
+      <c r="B69" t="s">
+        <v>328</v>
+      </c>
+      <c r="C69" t="s">
+        <v>381</v>
+      </c>
+      <c r="D69" t="s">
+        <v>438</v>
+      </c>
+      <c r="E69" t="s">
+        <v>390</v>
+      </c>
+      <c r="F69" t="s">
+        <v>15</v>
+      </c>
+      <c r="G69" t="s">
+        <v>439</v>
+      </c>
+      <c r="H69" t="s">
+        <v>440</v>
+      </c>
+      <c r="I69" t="s">
+        <v>441</v>
+      </c>
+      <c r="J69" t="s">
+        <v>442</v>
+      </c>
+      <c r="K69" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11">
+      <c r="A70" t="s">
+        <v>444</v>
+      </c>
+      <c r="B70" t="s">
+        <v>328</v>
+      </c>
+      <c r="C70" t="s">
+        <v>381</v>
+      </c>
+      <c r="D70" t="s">
+        <v>445</v>
+      </c>
+      <c r="F70" t="s">
+        <v>15</v>
+      </c>
+      <c r="G70" t="s">
+        <v>446</v>
+      </c>
+      <c r="H70" t="s">
+        <v>447</v>
+      </c>
+      <c r="I70" t="s">
+        <v>447</v>
+      </c>
+      <c r="J70" t="s">
+        <v>448</v>
+      </c>
+      <c r="K70" t="s">
+        <v>449</v>
       </c>
     </row>
   </sheetData>
@@ -4819,7 +5173,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39EA8986-82CF-4065-B488-659BF03572F5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{944AE346-DC81-4D40-8AA3-E0FF73D9CB6F}">
   <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
@@ -4841,22 +5195,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>405</v>
+        <v>450</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>406</v>
+        <v>451</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>407</v>
+        <v>452</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>408</v>
+        <v>453</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>409</v>
+        <v>454</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>410</v>
+        <v>455</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
@@ -4873,645 +5227,645 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>411</v>
+        <v>456</v>
       </c>
       <c r="B2" t="s">
-        <v>412</v>
+        <v>457</v>
       </c>
       <c r="C2" t="s">
-        <v>413</v>
+        <v>458</v>
       </c>
       <c r="D2" t="s">
-        <v>414</v>
+        <v>459</v>
       </c>
       <c r="E2" t="s">
-        <v>415</v>
+        <v>460</v>
       </c>
       <c r="F2" t="s">
-        <v>416</v>
+        <v>461</v>
       </c>
       <c r="G2" t="s">
-        <v>417</v>
+        <v>462</v>
       </c>
       <c r="H2" t="s">
-        <v>418</v>
+        <v>463</v>
       </c>
       <c r="I2" t="s">
-        <v>418</v>
+        <v>463</v>
       </c>
       <c r="J2" t="s">
-        <v>419</v>
+        <v>464</v>
       </c>
       <c r="K2" t="s">
-        <v>420</v>
+        <v>465</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>421</v>
+        <v>466</v>
       </c>
       <c r="B3" t="s">
-        <v>412</v>
+        <v>457</v>
       </c>
       <c r="C3" t="s">
-        <v>413</v>
+        <v>458</v>
       </c>
       <c r="D3" t="s">
-        <v>422</v>
+        <v>467</v>
       </c>
       <c r="E3" t="s">
-        <v>415</v>
+        <v>460</v>
       </c>
       <c r="F3" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H3" t="s">
-        <v>424</v>
+        <v>469</v>
       </c>
       <c r="I3" t="s">
-        <v>424</v>
+        <v>469</v>
       </c>
       <c r="J3" t="s">
-        <v>425</v>
+        <v>470</v>
       </c>
       <c r="K3" t="s">
-        <v>426</v>
+        <v>471</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>427</v>
+        <v>472</v>
       </c>
       <c r="B4" t="s">
-        <v>412</v>
+        <v>457</v>
       </c>
       <c r="C4" t="s">
-        <v>413</v>
+        <v>458</v>
       </c>
       <c r="D4" t="s">
-        <v>428</v>
+        <v>473</v>
       </c>
       <c r="E4" t="s">
-        <v>415</v>
+        <v>460</v>
       </c>
       <c r="F4" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H4" t="s">
-        <v>429</v>
+        <v>474</v>
       </c>
       <c r="I4" t="s">
-        <v>429</v>
+        <v>474</v>
       </c>
       <c r="J4" t="s">
-        <v>430</v>
+        <v>475</v>
       </c>
       <c r="K4" t="s">
-        <v>431</v>
+        <v>476</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>432</v>
+        <v>477</v>
       </c>
       <c r="B5" t="s">
-        <v>412</v>
+        <v>457</v>
       </c>
       <c r="C5" t="s">
-        <v>413</v>
+        <v>458</v>
       </c>
       <c r="D5" t="s">
-        <v>433</v>
+        <v>478</v>
       </c>
       <c r="E5" t="s">
-        <v>415</v>
+        <v>460</v>
       </c>
       <c r="F5" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H5" t="s">
-        <v>434</v>
+        <v>479</v>
       </c>
       <c r="I5" t="s">
-        <v>434</v>
+        <v>479</v>
       </c>
       <c r="J5" t="s">
-        <v>435</v>
+        <v>480</v>
       </c>
       <c r="K5" t="s">
-        <v>436</v>
+        <v>481</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>437</v>
+        <v>482</v>
       </c>
       <c r="B6" t="s">
-        <v>412</v>
+        <v>457</v>
       </c>
       <c r="C6" t="s">
-        <v>413</v>
+        <v>458</v>
       </c>
       <c r="D6" t="s">
-        <v>438</v>
+        <v>483</v>
       </c>
       <c r="E6" t="s">
-        <v>415</v>
+        <v>460</v>
       </c>
       <c r="F6" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H6" t="s">
-        <v>439</v>
+        <v>484</v>
       </c>
       <c r="I6" t="s">
-        <v>439</v>
+        <v>484</v>
       </c>
       <c r="J6" t="s">
-        <v>440</v>
+        <v>485</v>
       </c>
       <c r="K6" t="s">
-        <v>441</v>
+        <v>486</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>442</v>
+        <v>487</v>
       </c>
       <c r="B7" t="s">
-        <v>412</v>
+        <v>457</v>
       </c>
       <c r="C7" t="s">
-        <v>413</v>
+        <v>458</v>
       </c>
       <c r="D7" t="s">
-        <v>443</v>
+        <v>488</v>
       </c>
       <c r="E7" t="s">
-        <v>444</v>
+        <v>489</v>
       </c>
       <c r="F7" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H7" t="s">
-        <v>445</v>
+        <v>490</v>
       </c>
       <c r="I7" t="s">
-        <v>445</v>
+        <v>490</v>
       </c>
       <c r="J7" t="s">
-        <v>446</v>
+        <v>491</v>
       </c>
       <c r="K7" t="s">
-        <v>447</v>
+        <v>492</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>448</v>
+        <v>493</v>
       </c>
       <c r="B8" t="s">
-        <v>412</v>
+        <v>457</v>
       </c>
       <c r="C8" t="s">
-        <v>413</v>
+        <v>458</v>
       </c>
       <c r="D8" t="s">
-        <v>449</v>
+        <v>494</v>
       </c>
       <c r="E8" t="s">
-        <v>415</v>
+        <v>460</v>
       </c>
       <c r="F8" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H8" t="s">
-        <v>450</v>
+        <v>495</v>
       </c>
       <c r="I8" t="s">
-        <v>451</v>
+        <v>496</v>
       </c>
       <c r="J8" t="s">
-        <v>452</v>
+        <v>497</v>
       </c>
       <c r="K8" t="s">
-        <v>453</v>
+        <v>498</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>454</v>
+        <v>499</v>
       </c>
       <c r="B9" t="s">
-        <v>412</v>
+        <v>457</v>
       </c>
       <c r="C9" t="s">
-        <v>413</v>
+        <v>458</v>
       </c>
       <c r="D9" t="s">
-        <v>455</v>
+        <v>500</v>
       </c>
       <c r="E9" t="s">
-        <v>456</v>
+        <v>501</v>
       </c>
       <c r="F9" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H9" t="s">
-        <v>457</v>
+        <v>502</v>
       </c>
       <c r="I9" t="s">
-        <v>458</v>
+        <v>503</v>
       </c>
       <c r="J9" t="s">
-        <v>459</v>
+        <v>504</v>
       </c>
       <c r="K9" t="s">
-        <v>460</v>
+        <v>505</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>461</v>
+        <v>506</v>
       </c>
       <c r="B10" t="s">
-        <v>412</v>
+        <v>457</v>
       </c>
       <c r="C10" t="s">
-        <v>413</v>
+        <v>458</v>
       </c>
       <c r="D10" t="s">
-        <v>462</v>
+        <v>507</v>
       </c>
       <c r="E10" t="s">
-        <v>463</v>
+        <v>508</v>
       </c>
       <c r="F10" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H10" t="s">
-        <v>464</v>
+        <v>509</v>
       </c>
       <c r="I10" t="s">
-        <v>465</v>
+        <v>510</v>
       </c>
       <c r="J10" t="s">
-        <v>466</v>
+        <v>511</v>
       </c>
       <c r="K10" t="s">
-        <v>467</v>
+        <v>512</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>468</v>
+        <v>513</v>
       </c>
       <c r="B11" t="s">
-        <v>412</v>
+        <v>457</v>
       </c>
       <c r="C11" t="s">
-        <v>413</v>
+        <v>458</v>
       </c>
       <c r="D11" t="s">
-        <v>469</v>
+        <v>514</v>
       </c>
       <c r="E11" t="s">
-        <v>456</v>
+        <v>501</v>
       </c>
       <c r="F11" t="s">
-        <v>416</v>
+        <v>461</v>
       </c>
       <c r="H11" t="s">
-        <v>470</v>
+        <v>515</v>
       </c>
       <c r="I11" t="s">
-        <v>471</v>
+        <v>516</v>
       </c>
       <c r="J11" t="s">
-        <v>472</v>
+        <v>517</v>
       </c>
       <c r="K11" t="s">
-        <v>473</v>
+        <v>518</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>474</v>
+        <v>519</v>
       </c>
       <c r="B12" t="s">
-        <v>412</v>
+        <v>457</v>
       </c>
       <c r="C12" t="s">
-        <v>413</v>
+        <v>458</v>
       </c>
       <c r="D12" t="s">
-        <v>475</v>
+        <v>520</v>
       </c>
       <c r="E12" t="s">
-        <v>415</v>
+        <v>460</v>
       </c>
       <c r="F12" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H12" t="s">
-        <v>290</v>
+        <v>317</v>
       </c>
       <c r="I12" t="s">
-        <v>476</v>
+        <v>521</v>
       </c>
       <c r="J12" t="s">
-        <v>477</v>
+        <v>522</v>
       </c>
       <c r="K12" t="s">
-        <v>478</v>
+        <v>523</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>479</v>
+        <v>524</v>
       </c>
       <c r="B13" t="s">
-        <v>480</v>
+        <v>525</v>
       </c>
       <c r="C13" t="s">
-        <v>481</v>
+        <v>526</v>
       </c>
       <c r="D13" t="s">
-        <v>482</v>
+        <v>527</v>
       </c>
       <c r="E13" t="s">
-        <v>456</v>
+        <v>501</v>
       </c>
       <c r="F13" t="s">
-        <v>416</v>
+        <v>461</v>
       </c>
       <c r="H13" t="s">
-        <v>483</v>
+        <v>528</v>
       </c>
       <c r="I13" t="s">
-        <v>484</v>
+        <v>529</v>
       </c>
       <c r="J13" t="s">
-        <v>485</v>
+        <v>530</v>
       </c>
       <c r="K13" t="s">
-        <v>486</v>
+        <v>531</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>487</v>
+        <v>532</v>
       </c>
       <c r="B14" t="s">
-        <v>480</v>
+        <v>525</v>
       </c>
       <c r="C14" t="s">
-        <v>481</v>
+        <v>526</v>
       </c>
       <c r="D14" t="s">
-        <v>488</v>
+        <v>533</v>
       </c>
       <c r="E14" t="s">
-        <v>415</v>
+        <v>460</v>
       </c>
       <c r="F14" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H14" t="s">
-        <v>489</v>
+        <v>534</v>
       </c>
       <c r="I14" t="s">
-        <v>489</v>
+        <v>534</v>
       </c>
       <c r="J14" t="s">
-        <v>490</v>
+        <v>535</v>
       </c>
       <c r="K14" t="s">
-        <v>491</v>
+        <v>536</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>492</v>
+        <v>537</v>
       </c>
       <c r="B15" t="s">
-        <v>480</v>
+        <v>525</v>
       </c>
       <c r="C15" t="s">
-        <v>481</v>
+        <v>526</v>
       </c>
       <c r="D15" t="s">
-        <v>493</v>
+        <v>538</v>
       </c>
       <c r="E15" t="s">
-        <v>444</v>
+        <v>489</v>
       </c>
       <c r="F15" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H15" t="s">
-        <v>494</v>
+        <v>539</v>
       </c>
       <c r="I15" t="s">
-        <v>495</v>
+        <v>540</v>
       </c>
       <c r="J15" t="s">
-        <v>496</v>
+        <v>541</v>
       </c>
       <c r="K15" t="s">
-        <v>497</v>
+        <v>542</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>498</v>
+        <v>543</v>
       </c>
       <c r="B16" t="s">
-        <v>480</v>
+        <v>525</v>
       </c>
       <c r="C16" t="s">
-        <v>481</v>
+        <v>526</v>
       </c>
       <c r="D16" t="s">
-        <v>499</v>
+        <v>544</v>
       </c>
       <c r="E16" t="s">
-        <v>415</v>
+        <v>460</v>
       </c>
       <c r="F16" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H16" t="s">
-        <v>500</v>
+        <v>545</v>
       </c>
       <c r="I16" t="s">
-        <v>501</v>
+        <v>546</v>
       </c>
       <c r="J16" t="s">
-        <v>502</v>
+        <v>547</v>
       </c>
       <c r="K16" t="s">
-        <v>503</v>
+        <v>548</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>504</v>
+        <v>549</v>
       </c>
       <c r="B17" t="s">
-        <v>480</v>
+        <v>525</v>
       </c>
       <c r="C17" t="s">
-        <v>481</v>
+        <v>526</v>
       </c>
       <c r="D17" t="s">
-        <v>505</v>
+        <v>550</v>
       </c>
       <c r="E17" t="s">
-        <v>415</v>
+        <v>460</v>
       </c>
       <c r="F17" t="s">
-        <v>416</v>
+        <v>461</v>
       </c>
       <c r="H17" t="s">
-        <v>506</v>
+        <v>551</v>
       </c>
       <c r="I17" t="s">
-        <v>507</v>
+        <v>552</v>
       </c>
       <c r="J17" t="s">
-        <v>508</v>
+        <v>553</v>
       </c>
       <c r="K17" t="s">
-        <v>509</v>
+        <v>554</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>510</v>
+        <v>555</v>
       </c>
       <c r="B18" t="s">
-        <v>480</v>
+        <v>525</v>
       </c>
       <c r="C18" t="s">
-        <v>481</v>
+        <v>526</v>
       </c>
       <c r="D18" t="s">
-        <v>511</v>
+        <v>556</v>
       </c>
       <c r="E18" t="s">
-        <v>444</v>
+        <v>489</v>
       </c>
       <c r="F18" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H18" t="s">
-        <v>512</v>
+        <v>557</v>
       </c>
       <c r="I18" t="s">
-        <v>513</v>
+        <v>558</v>
       </c>
       <c r="J18" t="s">
-        <v>514</v>
+        <v>559</v>
       </c>
       <c r="K18" t="s">
-        <v>515</v>
+        <v>560</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" t="s">
-        <v>516</v>
+        <v>561</v>
       </c>
       <c r="B19" t="s">
-        <v>480</v>
+        <v>525</v>
       </c>
       <c r="C19" t="s">
-        <v>517</v>
+        <v>562</v>
       </c>
       <c r="D19" t="s">
-        <v>518</v>
+        <v>563</v>
       </c>
       <c r="E19" t="s">
-        <v>415</v>
+        <v>460</v>
       </c>
       <c r="F19" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H19" t="s">
-        <v>519</v>
+        <v>564</v>
       </c>
       <c r="I19" t="s">
-        <v>519</v>
+        <v>564</v>
       </c>
       <c r="J19" t="s">
-        <v>520</v>
+        <v>565</v>
       </c>
       <c r="K19" t="s">
-        <v>521</v>
+        <v>566</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>522</v>
+        <v>567</v>
       </c>
       <c r="B20" t="s">
-        <v>480</v>
+        <v>525</v>
       </c>
       <c r="C20" t="s">
-        <v>517</v>
+        <v>562</v>
       </c>
       <c r="D20" t="s">
-        <v>523</v>
+        <v>568</v>
       </c>
       <c r="E20" t="s">
-        <v>444</v>
+        <v>489</v>
       </c>
       <c r="F20" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H20" t="s">
-        <v>524</v>
+        <v>569</v>
       </c>
       <c r="I20" t="s">
-        <v>525</v>
+        <v>570</v>
       </c>
       <c r="J20" t="s">
-        <v>526</v>
+        <v>571</v>
       </c>
       <c r="K20" t="s">
-        <v>527</v>
+        <v>572</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>528</v>
+        <v>573</v>
       </c>
       <c r="B21" t="s">
-        <v>480</v>
+        <v>525</v>
       </c>
       <c r="C21" t="s">
-        <v>517</v>
+        <v>562</v>
       </c>
       <c r="D21" t="s">
-        <v>529</v>
+        <v>574</v>
       </c>
       <c r="E21" t="s">
-        <v>444</v>
+        <v>489</v>
       </c>
       <c r="F21" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
       <c r="H21" t="s">
-        <v>530</v>
+        <v>575</v>
       </c>
       <c r="I21" t="s">
-        <v>531</v>
+        <v>576</v>
       </c>
       <c r="J21" t="s">
-        <v>532</v>
+        <v>577</v>
       </c>
       <c r="K21" t="s">
-        <v>533</v>
+        <v>578</v>
       </c>
     </row>
   </sheetData>
@@ -5521,7 +5875,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43136E99-29D0-4A68-B90F-6C25D8CE8256}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F865740-48E8-4E73-B837-DAD528B3468E}">
   <dimension ref="A1:E41"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
@@ -5537,696 +5891,696 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>534</v>
+        <v>579</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>535</v>
+        <v>580</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>536</v>
+        <v>581</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>537</v>
+        <v>582</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>538</v>
+        <v>583</v>
       </c>
       <c r="B2" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C2" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D2" t="s">
-        <v>541</v>
+        <v>586</v>
       </c>
       <c r="E2" t="s">
-        <v>542</v>
+        <v>587</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>543</v>
+        <v>588</v>
       </c>
       <c r="B3" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C3" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D3" t="s">
-        <v>544</v>
+        <v>589</v>
       </c>
       <c r="E3" t="s">
-        <v>545</v>
+        <v>590</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>546</v>
+        <v>591</v>
       </c>
       <c r="B4" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C4" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D4" t="s">
-        <v>547</v>
+        <v>592</v>
       </c>
       <c r="E4" t="s">
-        <v>548</v>
+        <v>593</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>549</v>
+        <v>594</v>
       </c>
       <c r="B5" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C5" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D5" t="s">
-        <v>550</v>
+        <v>595</v>
       </c>
       <c r="E5" t="s">
-        <v>551</v>
+        <v>596</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>552</v>
+        <v>597</v>
       </c>
       <c r="B6" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C6" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D6" t="s">
-        <v>553</v>
+        <v>598</v>
       </c>
       <c r="E6" t="s">
-        <v>554</v>
+        <v>599</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>555</v>
+        <v>600</v>
       </c>
       <c r="B7" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C7" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D7" t="s">
-        <v>556</v>
+        <v>601</v>
       </c>
       <c r="E7" t="s">
-        <v>557</v>
+        <v>602</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>558</v>
+        <v>603</v>
       </c>
       <c r="B8" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C8" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D8" t="s">
-        <v>559</v>
+        <v>604</v>
       </c>
       <c r="E8" t="s">
-        <v>560</v>
+        <v>605</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>561</v>
+        <v>606</v>
       </c>
       <c r="B9" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C9" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D9" t="s">
-        <v>562</v>
+        <v>607</v>
       </c>
       <c r="E9" t="s">
-        <v>563</v>
+        <v>608</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>564</v>
+        <v>609</v>
       </c>
       <c r="B10" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C10" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D10" t="s">
-        <v>565</v>
+        <v>610</v>
       </c>
       <c r="E10" t="s">
-        <v>566</v>
+        <v>611</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>567</v>
+        <v>612</v>
       </c>
       <c r="B11" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C11" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D11" t="s">
-        <v>568</v>
+        <v>613</v>
       </c>
       <c r="E11" t="s">
-        <v>569</v>
+        <v>614</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>570</v>
+        <v>615</v>
       </c>
       <c r="B12" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C12" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D12" t="s">
-        <v>571</v>
+        <v>616</v>
       </c>
       <c r="E12" t="s">
-        <v>572</v>
+        <v>617</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>573</v>
+        <v>618</v>
       </c>
       <c r="B13" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C13" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D13" t="s">
-        <v>574</v>
+        <v>619</v>
       </c>
       <c r="E13" t="s">
-        <v>575</v>
+        <v>620</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>576</v>
+        <v>621</v>
       </c>
       <c r="B14" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C14" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D14" t="s">
-        <v>577</v>
+        <v>622</v>
       </c>
       <c r="E14" t="s">
-        <v>578</v>
+        <v>623</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>579</v>
+        <v>624</v>
       </c>
       <c r="B15" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C15" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D15" t="s">
-        <v>580</v>
+        <v>625</v>
       </c>
       <c r="E15" t="s">
-        <v>581</v>
+        <v>626</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>582</v>
+        <v>627</v>
       </c>
       <c r="B16" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C16" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D16" t="s">
-        <v>583</v>
+        <v>628</v>
       </c>
       <c r="E16" t="s">
-        <v>584</v>
+        <v>629</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
+        <v>630</v>
+      </c>
+      <c r="B17" t="s">
+        <v>584</v>
+      </c>
+      <c r="C17" t="s">
         <v>585</v>
       </c>
-      <c r="B17" t="s">
-        <v>539</v>
-      </c>
-      <c r="C17" t="s">
-        <v>540</v>
-      </c>
       <c r="D17" t="s">
-        <v>586</v>
+        <v>631</v>
       </c>
       <c r="E17" t="s">
-        <v>587</v>
+        <v>632</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>588</v>
+        <v>633</v>
       </c>
       <c r="B18" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C18" t="s">
-        <v>589</v>
+        <v>634</v>
       </c>
       <c r="D18" t="s">
-        <v>590</v>
+        <v>635</v>
       </c>
       <c r="E18" t="s">
-        <v>591</v>
+        <v>636</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>592</v>
+        <v>637</v>
       </c>
       <c r="B19" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C19" t="s">
-        <v>589</v>
+        <v>634</v>
       </c>
       <c r="D19" t="s">
-        <v>593</v>
+        <v>638</v>
       </c>
       <c r="E19" t="s">
-        <v>594</v>
+        <v>639</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>595</v>
+        <v>640</v>
       </c>
       <c r="B20" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C20" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D20" t="s">
-        <v>596</v>
+        <v>641</v>
       </c>
       <c r="E20" t="s">
-        <v>597</v>
+        <v>642</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>598</v>
+        <v>643</v>
       </c>
       <c r="B21" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C21" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D21" t="s">
-        <v>599</v>
+        <v>644</v>
       </c>
       <c r="E21" t="s">
-        <v>600</v>
+        <v>645</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>601</v>
+        <v>646</v>
       </c>
       <c r="B22" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C22" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D22" t="s">
-        <v>602</v>
+        <v>647</v>
       </c>
       <c r="E22" t="s">
-        <v>603</v>
+        <v>648</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>604</v>
+        <v>649</v>
       </c>
       <c r="B23" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C23" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D23" t="s">
-        <v>605</v>
+        <v>650</v>
       </c>
       <c r="E23" t="s">
-        <v>606</v>
+        <v>651</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>607</v>
+        <v>652</v>
       </c>
       <c r="B24" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C24" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D24" t="s">
-        <v>608</v>
+        <v>653</v>
       </c>
       <c r="E24" t="s">
-        <v>609</v>
+        <v>654</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>610</v>
+        <v>655</v>
       </c>
       <c r="B25" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C25" t="s">
-        <v>611</v>
+        <v>656</v>
       </c>
       <c r="D25" t="s">
-        <v>612</v>
+        <v>657</v>
       </c>
       <c r="E25" t="s">
-        <v>613</v>
+        <v>658</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>614</v>
+        <v>659</v>
       </c>
       <c r="B26" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C26" t="s">
-        <v>589</v>
+        <v>634</v>
       </c>
       <c r="D26" t="s">
-        <v>615</v>
+        <v>660</v>
       </c>
       <c r="E26" t="s">
-        <v>616</v>
+        <v>661</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>617</v>
+        <v>662</v>
       </c>
       <c r="B27" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C27" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D27" t="s">
-        <v>618</v>
+        <v>663</v>
       </c>
       <c r="E27" t="s">
-        <v>619</v>
+        <v>664</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>620</v>
+        <v>665</v>
       </c>
       <c r="B28" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C28" t="s">
-        <v>589</v>
+        <v>634</v>
       </c>
       <c r="D28" t="s">
-        <v>621</v>
+        <v>666</v>
       </c>
       <c r="E28" t="s">
-        <v>622</v>
+        <v>667</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>623</v>
+        <v>668</v>
       </c>
       <c r="B29" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="C29" t="s">
-        <v>611</v>
+        <v>656</v>
       </c>
       <c r="D29" t="s">
-        <v>624</v>
+        <v>669</v>
       </c>
       <c r="E29" t="s">
-        <v>625</v>
+        <v>670</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>626</v>
+        <v>671</v>
       </c>
       <c r="B30" t="s">
-        <v>627</v>
+        <v>672</v>
       </c>
       <c r="C30" t="s">
-        <v>589</v>
+        <v>634</v>
       </c>
       <c r="D30" t="s">
-        <v>628</v>
+        <v>673</v>
       </c>
       <c r="E30" t="s">
-        <v>629</v>
+        <v>674</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>630</v>
+        <v>675</v>
       </c>
       <c r="B31" t="s">
-        <v>627</v>
+        <v>672</v>
       </c>
       <c r="C31" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D31" t="s">
-        <v>631</v>
+        <v>676</v>
       </c>
       <c r="E31" t="s">
-        <v>632</v>
+        <v>677</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>633</v>
+        <v>678</v>
       </c>
       <c r="B32" t="s">
-        <v>627</v>
+        <v>672</v>
       </c>
       <c r="C32" t="s">
-        <v>589</v>
+        <v>634</v>
       </c>
       <c r="D32" t="s">
-        <v>634</v>
+        <v>679</v>
       </c>
       <c r="E32" t="s">
-        <v>635</v>
+        <v>680</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>636</v>
+        <v>681</v>
       </c>
       <c r="B33" t="s">
-        <v>627</v>
+        <v>672</v>
       </c>
       <c r="C33" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D33" t="s">
-        <v>637</v>
+        <v>682</v>
       </c>
       <c r="E33" t="s">
-        <v>638</v>
+        <v>683</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>639</v>
+        <v>684</v>
       </c>
       <c r="B34" t="s">
-        <v>640</v>
+        <v>685</v>
       </c>
       <c r="C34" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D34" t="s">
-        <v>641</v>
+        <v>686</v>
       </c>
       <c r="E34" t="s">
-        <v>642</v>
+        <v>687</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>643</v>
+        <v>688</v>
       </c>
       <c r="B35" t="s">
-        <v>640</v>
+        <v>685</v>
       </c>
       <c r="C35" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D35" t="s">
-        <v>644</v>
+        <v>689</v>
       </c>
       <c r="E35" t="s">
-        <v>645</v>
+        <v>690</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>646</v>
+        <v>691</v>
       </c>
       <c r="B36" t="s">
-        <v>640</v>
+        <v>685</v>
       </c>
       <c r="C36" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D36" t="s">
-        <v>647</v>
+        <v>692</v>
       </c>
       <c r="E36" t="s">
-        <v>648</v>
+        <v>693</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>649</v>
+        <v>694</v>
       </c>
       <c r="B37" t="s">
-        <v>640</v>
+        <v>685</v>
       </c>
       <c r="C37" t="s">
-        <v>589</v>
+        <v>634</v>
       </c>
       <c r="D37" t="s">
-        <v>650</v>
+        <v>695</v>
       </c>
       <c r="E37" t="s">
-        <v>651</v>
+        <v>696</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>652</v>
+        <v>697</v>
       </c>
       <c r="B38" t="s">
-        <v>640</v>
+        <v>685</v>
       </c>
       <c r="C38" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D38" t="s">
-        <v>653</v>
+        <v>698</v>
       </c>
       <c r="E38" t="s">
-        <v>654</v>
+        <v>699</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>655</v>
+        <v>700</v>
       </c>
       <c r="B39" t="s">
-        <v>656</v>
+        <v>701</v>
       </c>
       <c r="C39" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
       <c r="D39" t="s">
-        <v>657</v>
+        <v>702</v>
       </c>
       <c r="E39" t="s">
-        <v>658</v>
+        <v>703</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>659</v>
+        <v>704</v>
       </c>
       <c r="B40" t="s">
-        <v>656</v>
+        <v>701</v>
       </c>
       <c r="C40" t="s">
-        <v>589</v>
+        <v>634</v>
       </c>
       <c r="D40" t="s">
-        <v>660</v>
+        <v>705</v>
       </c>
       <c r="E40" t="s">
-        <v>661</v>
+        <v>706</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>662</v>
+        <v>707</v>
       </c>
       <c r="B41" t="s">
-        <v>656</v>
+        <v>701</v>
       </c>
       <c r="C41" t="s">
-        <v>589</v>
+        <v>634</v>
       </c>
       <c r="D41" t="s">
-        <v>663</v>
+        <v>708</v>
       </c>
       <c r="E41" t="s">
-        <v>664</v>
+        <v>709</v>
       </c>
     </row>
   </sheetData>
@@ -6236,7 +6590,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F552A4D2-FB82-4063-862C-E2CD3384FC8D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99BBABED-2C5B-4190-B266-EE29E03ACB04}">
   <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
@@ -6255,363 +6609,363 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>665</v>
+        <v>710</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>666</v>
+        <v>711</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>667</v>
+        <v>712</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>668</v>
+        <v>713</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>669</v>
+        <v>714</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>670</v>
+        <v>715</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>671</v>
+        <v>716</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>672</v>
+        <v>717</v>
       </c>
       <c r="B2" t="s">
-        <v>673</v>
+        <v>718</v>
       </c>
       <c r="C2" t="s">
-        <v>674</v>
+        <v>719</v>
       </c>
       <c r="D2" t="s">
-        <v>675</v>
+        <v>720</v>
       </c>
       <c r="E2" t="s">
-        <v>676</v>
+        <v>721</v>
       </c>
       <c r="F2" t="s">
-        <v>677</v>
+        <v>722</v>
       </c>
       <c r="G2" t="s">
-        <v>678</v>
+        <v>723</v>
       </c>
       <c r="H2" t="s">
-        <v>679</v>
+        <v>724</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>680</v>
+        <v>725</v>
       </c>
       <c r="B3" t="s">
-        <v>673</v>
+        <v>718</v>
       </c>
       <c r="C3" t="s">
-        <v>681</v>
+        <v>726</v>
       </c>
       <c r="D3" t="s">
-        <v>682</v>
+        <v>727</v>
       </c>
       <c r="E3" t="s">
-        <v>683</v>
+        <v>728</v>
       </c>
       <c r="F3" t="s">
-        <v>684</v>
+        <v>729</v>
       </c>
       <c r="G3" t="s">
-        <v>685</v>
+        <v>730</v>
       </c>
       <c r="H3" t="s">
-        <v>679</v>
+        <v>724</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>686</v>
+        <v>731</v>
       </c>
       <c r="B4" t="s">
-        <v>673</v>
+        <v>718</v>
       </c>
       <c r="C4" t="s">
-        <v>687</v>
+        <v>732</v>
       </c>
       <c r="D4" t="s">
-        <v>682</v>
+        <v>727</v>
       </c>
       <c r="E4" t="s">
-        <v>688</v>
+        <v>733</v>
       </c>
       <c r="F4" t="s">
-        <v>689</v>
+        <v>734</v>
       </c>
       <c r="G4" t="s">
-        <v>690</v>
+        <v>735</v>
       </c>
       <c r="H4" t="s">
-        <v>679</v>
+        <v>724</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>691</v>
+        <v>736</v>
       </c>
       <c r="B5" t="s">
-        <v>673</v>
+        <v>718</v>
       </c>
       <c r="C5" t="s">
-        <v>692</v>
+        <v>737</v>
       </c>
       <c r="D5" t="s">
-        <v>693</v>
+        <v>738</v>
       </c>
       <c r="E5" t="s">
-        <v>694</v>
+        <v>739</v>
       </c>
       <c r="F5" t="s">
-        <v>695</v>
+        <v>740</v>
       </c>
       <c r="G5" t="s">
-        <v>696</v>
+        <v>741</v>
       </c>
       <c r="H5" t="s">
-        <v>697</v>
+        <v>742</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>698</v>
+        <v>743</v>
       </c>
       <c r="B6" t="s">
-        <v>673</v>
+        <v>718</v>
       </c>
       <c r="C6" t="s">
-        <v>699</v>
+        <v>744</v>
       </c>
       <c r="D6" t="s">
-        <v>675</v>
+        <v>720</v>
       </c>
       <c r="E6" t="s">
-        <v>700</v>
+        <v>745</v>
       </c>
       <c r="F6" t="s">
-        <v>701</v>
+        <v>746</v>
       </c>
       <c r="G6" t="s">
-        <v>702</v>
+        <v>747</v>
       </c>
       <c r="H6" t="s">
-        <v>703</v>
+        <v>748</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>704</v>
+        <v>749</v>
       </c>
       <c r="B7" t="s">
-        <v>673</v>
+        <v>718</v>
       </c>
       <c r="C7" t="s">
-        <v>705</v>
+        <v>750</v>
       </c>
       <c r="D7" t="s">
-        <v>706</v>
+        <v>751</v>
       </c>
       <c r="E7" t="s">
-        <v>707</v>
+        <v>752</v>
       </c>
       <c r="F7" t="s">
-        <v>708</v>
+        <v>753</v>
       </c>
       <c r="G7" t="s">
-        <v>709</v>
+        <v>754</v>
       </c>
       <c r="H7" t="s">
-        <v>710</v>
+        <v>755</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>711</v>
+        <v>756</v>
       </c>
       <c r="B8" t="s">
-        <v>712</v>
+        <v>757</v>
       </c>
       <c r="C8" t="s">
-        <v>713</v>
+        <v>758</v>
       </c>
       <c r="D8" t="s">
-        <v>675</v>
+        <v>720</v>
       </c>
       <c r="E8" t="s">
-        <v>714</v>
+        <v>759</v>
       </c>
       <c r="F8" t="s">
-        <v>715</v>
+        <v>760</v>
       </c>
       <c r="G8" t="s">
-        <v>716</v>
+        <v>761</v>
       </c>
       <c r="H8" t="s">
-        <v>717</v>
+        <v>762</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>718</v>
+        <v>763</v>
       </c>
       <c r="B9" t="s">
-        <v>712</v>
+        <v>757</v>
       </c>
       <c r="C9" t="s">
-        <v>719</v>
+        <v>764</v>
       </c>
       <c r="D9" t="s">
-        <v>675</v>
+        <v>720</v>
       </c>
       <c r="E9" t="s">
-        <v>720</v>
+        <v>765</v>
       </c>
       <c r="F9" t="s">
-        <v>721</v>
+        <v>766</v>
       </c>
       <c r="G9" t="s">
-        <v>722</v>
+        <v>767</v>
       </c>
       <c r="H9" t="s">
-        <v>717</v>
+        <v>762</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>723</v>
+        <v>768</v>
       </c>
       <c r="B10" t="s">
-        <v>724</v>
+        <v>769</v>
       </c>
       <c r="C10" t="s">
-        <v>725</v>
+        <v>770</v>
       </c>
       <c r="D10" t="s">
-        <v>726</v>
+        <v>771</v>
       </c>
       <c r="E10" t="s">
-        <v>727</v>
+        <v>772</v>
       </c>
       <c r="F10" t="s">
-        <v>728</v>
+        <v>773</v>
       </c>
       <c r="G10" t="s">
-        <v>729</v>
+        <v>774</v>
       </c>
       <c r="H10" t="s">
-        <v>730</v>
+        <v>775</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>731</v>
+        <v>776</v>
       </c>
       <c r="B11" t="s">
-        <v>732</v>
+        <v>777</v>
       </c>
       <c r="C11" t="s">
-        <v>733</v>
+        <v>778</v>
       </c>
       <c r="D11" t="s">
-        <v>726</v>
+        <v>771</v>
       </c>
       <c r="E11" t="s">
-        <v>734</v>
+        <v>779</v>
       </c>
       <c r="F11" t="s">
-        <v>735</v>
+        <v>780</v>
       </c>
       <c r="G11" t="s">
-        <v>736</v>
+        <v>781</v>
       </c>
       <c r="H11" t="s">
-        <v>737</v>
+        <v>782</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>738</v>
+        <v>783</v>
       </c>
       <c r="B12" t="s">
-        <v>739</v>
+        <v>784</v>
       </c>
       <c r="C12" t="s">
-        <v>740</v>
+        <v>785</v>
       </c>
       <c r="D12" t="s">
-        <v>682</v>
+        <v>727</v>
       </c>
       <c r="E12" t="s">
-        <v>741</v>
+        <v>786</v>
       </c>
       <c r="F12" t="s">
-        <v>742</v>
+        <v>787</v>
       </c>
       <c r="G12" t="s">
-        <v>743</v>
+        <v>788</v>
       </c>
       <c r="H12" t="s">
-        <v>744</v>
+        <v>789</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>745</v>
+        <v>790</v>
       </c>
       <c r="B13" t="s">
-        <v>746</v>
+        <v>791</v>
       </c>
       <c r="C13" t="s">
-        <v>747</v>
+        <v>792</v>
       </c>
       <c r="D13" t="s">
-        <v>682</v>
+        <v>727</v>
       </c>
       <c r="E13" t="s">
-        <v>748</v>
+        <v>793</v>
       </c>
       <c r="F13" t="s">
-        <v>749</v>
+        <v>794</v>
       </c>
       <c r="G13" t="s">
-        <v>743</v>
+        <v>788</v>
       </c>
       <c r="H13" t="s">
-        <v>744</v>
+        <v>789</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>750</v>
+        <v>795</v>
       </c>
       <c r="B14" t="s">
-        <v>751</v>
+        <v>796</v>
       </c>
       <c r="C14" t="s">
-        <v>752</v>
+        <v>797</v>
       </c>
       <c r="D14" t="s">
-        <v>726</v>
+        <v>771</v>
       </c>
       <c r="E14" t="s">
-        <v>753</v>
+        <v>798</v>
       </c>
       <c r="F14" t="s">
-        <v>754</v>
+        <v>799</v>
       </c>
       <c r="G14" t="s">
-        <v>755</v>
+        <v>800</v>
       </c>
       <c r="H14" t="s">
-        <v>744</v>
+        <v>789</v>
       </c>
     </row>
   </sheetData>
@@ -6621,7 +6975,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A5589B3-69BE-4DFD-BEA2-5F5F989622B9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4956A2F2-F43A-4EF9-8583-5FD7E412FE5E}">
   <dimension ref="A1:Q8"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
@@ -6646,132 +7000,132 @@
   <sheetData>
     <row r="1" spans="1:17" ht="27.95" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>756</v>
+        <v>801</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>757</v>
+        <v>802</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>758</v>
+        <v>803</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>759</v>
+        <v>804</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>760</v>
+        <v>805</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>761</v>
+        <v>806</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>762</v>
+        <v>807</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>763</v>
+        <v>808</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>764</v>
+        <v>809</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>765</v>
+        <v>810</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>766</v>
+        <v>811</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>767</v>
+        <v>812</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>768</v>
+        <v>813</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>769</v>
+        <v>814</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>770</v>
+        <v>815</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>771</v>
+        <v>816</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>772</v>
+        <v>817</v>
       </c>
     </row>
     <row r="2" spans="1:17">
       <c r="A2" t="s">
-        <v>773</v>
+        <v>818</v>
       </c>
       <c r="B2" t="s">
-        <v>774</v>
+        <v>819</v>
       </c>
       <c r="C2" t="s">
-        <v>775</v>
+        <v>820</v>
       </c>
     </row>
     <row r="3" spans="1:17">
       <c r="A3" t="s">
-        <v>776</v>
+        <v>821</v>
       </c>
       <c r="B3" t="s">
-        <v>777</v>
+        <v>822</v>
       </c>
       <c r="C3" t="s">
-        <v>778</v>
+        <v>823</v>
       </c>
     </row>
     <row r="4" spans="1:17">
       <c r="A4" t="s">
-        <v>779</v>
+        <v>824</v>
       </c>
       <c r="B4" t="s">
-        <v>780</v>
+        <v>825</v>
       </c>
       <c r="C4" t="s">
-        <v>781</v>
+        <v>826</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" t="s">
-        <v>782</v>
+        <v>827</v>
       </c>
       <c r="B5" t="s">
-        <v>783</v>
+        <v>828</v>
       </c>
       <c r="C5" t="s">
-        <v>784</v>
+        <v>829</v>
       </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" t="s">
-        <v>785</v>
+        <v>830</v>
       </c>
       <c r="B6" t="s">
-        <v>786</v>
+        <v>831</v>
       </c>
       <c r="C6" t="s">
-        <v>787</v>
+        <v>832</v>
       </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" t="s">
-        <v>788</v>
+        <v>833</v>
       </c>
       <c r="B7" t="s">
-        <v>789</v>
+        <v>834</v>
       </c>
       <c r="C7" t="s">
-        <v>790</v>
+        <v>835</v>
       </c>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" t="s">
-        <v>791</v>
+        <v>836</v>
       </c>
       <c r="B8" t="s">
-        <v>792</v>
+        <v>837</v>
       </c>
       <c r="C8" t="s">
-        <v>793</v>
+        <v>838</v>
       </c>
     </row>
   </sheetData>
@@ -6781,7 +7135,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DC931DD-2A80-4CE3-BD8D-6EBD7186602B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DEBE49F-CFDD-4A45-A2DF-199F855CA052}">
   <dimension ref="A1:L1"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
@@ -6800,40 +7154,40 @@
   <sheetData>
     <row r="1" spans="1:12" ht="27.95" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>794</v>
+        <v>839</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>795</v>
+        <v>840</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>796</v>
+        <v>841</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>797</v>
+        <v>842</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>798</v>
+        <v>843</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>799</v>
+        <v>844</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>800</v>
+        <v>845</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>801</v>
+        <v>846</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>802</v>
+        <v>847</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>803</v>
+        <v>848</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>804</v>
+        <v>849</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>805</v>
+        <v>850</v>
       </c>
     </row>
   </sheetData>

</xml_diff>